<commit_message>
Full code for Figure 2
</commit_message>
<xml_diff>
--- a/data/MetalliCan/sites_for_lci.xlsx
+++ b/data/MetalliCan/sites_for_lci.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/regionalized_lci_mineral/data/MetalliCan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2961" documentId="13_ncr:1_{965BE886-D2C4-44D2-937F-E901E74C4ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E197436-D085-44A6-842A-AEDCFBD749A5}"/>
+  <xr:revisionPtr revIDLastSave="2964" documentId="13_ncr:1_{965BE886-D2C4-44D2-937F-E901E74C4ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4356C535-E0C5-4AF5-91ED-8686BD5CEE1B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{9D292A65-B8C8-46CC-8162-88CB3EA3ABC7}"/>
   </bookViews>
@@ -26779,6 +26779,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19A21E0B-06A8-4909-8999-69A6CC63874F}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AZ66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -26987,7 +26988,7 @@
         <v>1598</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
         <v>53</v>
       </c>
@@ -27107,7 +27108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>60</v>
       </c>
@@ -27231,7 +27232,7 @@
         <v>0.92040969387755101</v>
       </c>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>68</v>
       </c>
@@ -27325,7 +27326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>74</v>
       </c>
@@ -27452,7 +27453,7 @@
         <v>29.039084533163262</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>82</v>
       </c>
@@ -27564,7 +27565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>88</v>
       </c>
@@ -27682,7 +27683,7 @@
         <v>3.5165997959183577</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
         <v>524</v>
       </c>
@@ -27806,7 +27807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
         <v>526</v>
       </c>
@@ -27912,7 +27913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
         <v>109</v>
       </c>
@@ -28042,7 +28043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>527</v>
       </c>
@@ -28169,7 +28170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
         <v>116</v>
       </c>
@@ -28293,7 +28294,7 @@
         <v>24.008283837755101</v>
       </c>
     </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
         <v>125</v>
       </c>
@@ -28411,7 +28412,7 @@
         <v>2.7760508515306124</v>
       </c>
     </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>135</v>
       </c>
@@ -28532,7 +28533,7 @@
         <v>7.7388999209183664</v>
       </c>
     </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>139</v>
       </c>
@@ -28653,7 +28654,7 @@
         <v>0.12428704693877551</v>
       </c>
     </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
         <v>156</v>
       </c>
@@ -28774,7 +28775,7 @@
         <v>1.4536125510204081</v>
       </c>
     </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
         <v>161</v>
       </c>
@@ -28892,7 +28893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
         <v>529</v>
       </c>
@@ -29019,7 +29020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
         <v>167</v>
       </c>
@@ -29143,7 +29144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
         <v>173</v>
       </c>
@@ -29270,7 +29271,7 @@
         <v>4.4745421183166938</v>
       </c>
     </row>
-    <row r="21" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
         <v>180</v>
       </c>
@@ -29394,7 +29395,7 @@
         <v>4.476523630102041</v>
       </c>
     </row>
-    <row r="22" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
         <v>186</v>
       </c>
@@ -29521,7 +29522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
         <v>494</v>
       </c>
@@ -29624,7 +29625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>195</v>
       </c>
@@ -29742,7 +29743,7 @@
         <v>4.1704080612244905</v>
       </c>
     </row>
-    <row r="25" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
         <v>200</v>
       </c>
@@ -29863,7 +29864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
         <v>205</v>
       </c>
@@ -29987,7 +29988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
         <v>209</v>
       </c>
@@ -30105,7 +30106,7 @@
         <v>1.2201776096938775</v>
       </c>
     </row>
-    <row r="28" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
         <v>215</v>
       </c>
@@ -30232,7 +30233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:52" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:52" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
         <v>227</v>
       </c>
@@ -30356,7 +30357,7 @@
         <v>7.932820721938775</v>
       </c>
     </row>
-    <row r="30" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
         <v>232</v>
       </c>
@@ -30492,7 +30493,7 @@
         <v>9.8029027903061134</v>
       </c>
     </row>
-    <row r="31" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
         <v>534</v>
       </c>
@@ -30595,7 +30596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
         <v>239</v>
       </c>
@@ -30722,7 +30723,7 @@
         <v>7.253304461734694</v>
       </c>
     </row>
-    <row r="33" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
         <v>243</v>
       </c>
@@ -30840,7 +30841,7 @@
         <v>1.0473627551020408</v>
       </c>
     </row>
-    <row r="34" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="s">
         <v>249</v>
       </c>
@@ -30958,7 +30959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
         <v>267</v>
       </c>
@@ -31073,7 +31074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
         <v>277</v>
       </c>
@@ -31197,7 +31198,7 @@
         <v>12.41413683010194</v>
       </c>
     </row>
-    <row r="37" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
         <v>283</v>
       </c>
@@ -31321,7 +31322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
         <v>288</v>
       </c>
@@ -31448,7 +31449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
         <v>294</v>
       </c>
@@ -31566,7 +31567,7 @@
         <v>5.7128877551020407</v>
       </c>
     </row>
-    <row r="40" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
         <v>297</v>
       </c>
@@ -31687,7 +31688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
         <v>305</v>
       </c>
@@ -31805,7 +31806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
         <v>311</v>
       </c>
@@ -31929,7 +31930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
         <v>316</v>
       </c>
@@ -32020,7 +32021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
         <v>328</v>
       </c>
@@ -32141,7 +32142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
         <v>333</v>
       </c>
@@ -32268,7 +32269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
         <v>337</v>
       </c>
@@ -32386,7 +32387,7 @@
         <v>8.0534261301020305</v>
       </c>
     </row>
-    <row r="47" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
         <v>340</v>
       </c>
@@ -32516,7 +32517,7 @@
         <v>0.15869132653061224</v>
       </c>
     </row>
-    <row r="48" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
         <v>343</v>
       </c>
@@ -32643,7 +32644,7 @@
         <v>3.5769025000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
         <v>357</v>
       </c>
@@ -32755,7 +32756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
         <v>371</v>
       </c>
@@ -32882,7 +32883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
         <v>376</v>
       </c>
@@ -32988,7 +32989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
         <v>381</v>
       </c>
@@ -33103,7 +33104,7 @@
         <v>1.2269695984693878</v>
       </c>
     </row>
-    <row r="53" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
         <v>387</v>
       </c>
@@ -33200,7 +33201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
         <v>393</v>
       </c>
@@ -33321,7 +33322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="21" t="s">
         <v>533</v>
       </c>
@@ -33448,7 +33449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="21" t="s">
         <v>409</v>
       </c>
@@ -33542,7 +33543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="21" t="s">
         <v>419</v>
       </c>
@@ -33663,7 +33664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21" t="s">
         <v>423</v>
       </c>
@@ -33784,7 +33785,7 @@
         <v>4.1181668765306121</v>
       </c>
     </row>
-    <row r="59" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="21" t="s">
         <v>428</v>
       </c>
@@ -33963,14 +33964,17 @@
         <v>43726.856187782003</v>
       </c>
       <c r="Y60"/>
-      <c r="Z60"/>
+      <c r="Z60" s="34">
+        <f>AX60</f>
+        <v>10205.82</v>
+      </c>
       <c r="AA60">
         <f t="shared" si="5"/>
-        <v>43726.856187782003</v>
+        <v>33521.036187782003</v>
       </c>
       <c r="AB60" s="54">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0.69553984122603307</v>
       </c>
       <c r="AC60" s="34"/>
       <c r="AD60" s="34"/>
@@ -34085,14 +34089,17 @@
         <v>98408.871032543204</v>
       </c>
       <c r="Y61"/>
-      <c r="Z61"/>
+      <c r="Z61" s="34">
+        <f>AX61</f>
+        <v>7654.3649999999998</v>
+      </c>
       <c r="AA61">
         <f t="shared" si="5"/>
-        <v>98408.871032543204</v>
+        <v>90754.506032543199</v>
       </c>
       <c r="AB61" s="54">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>0.91565856799159639</v>
       </c>
       <c r="AC61" s="34"/>
       <c r="AD61" s="34"/>
@@ -34146,7 +34153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="21"/>
       <c r="B62" t="s">
         <v>273</v>
@@ -34265,7 +34272,7 @@
         <v>17.66760135719143</v>
       </c>
     </row>
-    <row r="63" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="21"/>
       <c r="B63" t="s">
         <v>191</v>
@@ -34378,7 +34385,7 @@
         <v>8.2519489795918357</v>
       </c>
     </row>
-    <row r="64" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="21"/>
       <c r="B64" t="s">
         <v>398</v>
@@ -34497,7 +34504,7 @@
         <v>4.2180154591836736</v>
       </c>
     </row>
-    <row r="65" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:52" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="21"/>
       <c r="B65" t="s">
         <v>361</v>
@@ -34619,7 +34626,7 @@
         <v>1.2300799484693878</v>
       </c>
     </row>
-    <row r="66" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:52" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="23"/>
       <c r="B66" s="24" t="s">
         <v>222</v>
@@ -34759,7 +34766,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ66" xr:uid="{19A21E0B-06A8-4909-8999-69A6CC63874F}"/>
+  <autoFilter ref="A1:AZ66" xr:uid="{19A21E0B-06A8-4909-8999-69A6CC63874F}">
+    <filterColumn colId="19">
+      <filters>
+        <filter val="Uranium"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>